<commit_message>
feat(run): complete G7 single-act outcome flow
</commit_message>
<xml_diff>
--- a/DataTables/Datas/battle.encounter.xlsx
+++ b/DataTables/Datas/battle.encounter.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R51fdf121ba8c456a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rd7215dda84ce4050"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -392,6 +392,7 @@
     <x:col min="1" max="1" width="8.75" customWidth="1"/>
     <x:col min="2" max="2" width="9.5" customWidth="1"/>
     <x:col min="3" max="3" width="20.75" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -404,6 +405,9 @@
       <x:c r="C1" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="D1" t="str">
+        <x:v>phase_two_behavior_group_id</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="s">
@@ -415,11 +419,15 @@
       <x:c r="C2" s="2" t="s">
         <x:v>5</x:v>
       </x:c>
+      <x:c r="D2" t="str">
+        <x:v>int?</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="s">
         <x:v>6</x:v>
       </x:c>
+      <x:c r="D3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="4" t="s">
@@ -431,6 +439,9 @@
       <x:c r="C4" s="4" t="s">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Phase two behavior group ID; 0 means none</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="B5" s="6">
@@ -438,6 +449,33 @@
       </x:c>
       <x:c r="C5" s="7" t="str">
         <x:v>2001,2002</x:v>
+      </x:c>
+      <x:c r="D5" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6"/>
+      <x:c r="B6" t="n">
+        <x:v>5101</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>2101</x:v>
+      </x:c>
+      <x:c r="D6" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7"/>
+      <x:c r="B7" t="n">
+        <x:v>5201</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>2201</x:v>
+      </x:c>
+      <x:c r="D7" t="n">
+        <x:v>6202</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>